<commit_message>
okazało sie że ja z dupy zrobiłem jeden punkt
i nie wiedziałem w etapie 1 już bylo zrobione user moze edytowac aktywną oferte
</commit_message>
<xml_diff>
--- a/sprzatando excel.xlsx
+++ b/sprzatando excel.xlsx
@@ -683,7 +683,7 @@
       </c>
       <c r="G7" s="3" t="n">
         <f aca="false">COUNTIF(C:E, TRUE())</f>
-        <v>9</v>
+        <v>10</v>
       </c>
     </row>
     <row r="8" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -746,7 +746,7 @@
       </c>
       <c r="G11" s="7" t="n">
         <f aca="false">G7*100/G3</f>
-        <v>36</v>
+        <v>40</v>
       </c>
     </row>
     <row r="12" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -911,8 +911,8 @@
         <v>0</v>
       </c>
       <c r="D19" s="1" t="b">
-        <f aca="false">FALSE()</f>
-        <v>0</v>
+        <f aca="false">TRUE()</f>
+        <v>1</v>
       </c>
       <c r="E19" s="1" t="b">
         <f aca="false">FALSE()</f>
@@ -974,7 +974,7 @@
         <f aca="false">FALSE()</f>
         <v>0</v>
       </c>
-      <c r="F23" s="0" t="s">
+      <c r="F23" s="1" t="s">
         <v>35</v>
       </c>
     </row>
@@ -994,7 +994,7 @@
         <f aca="false">FALSE()</f>
         <v>0</v>
       </c>
-      <c r="F24" s="0" t="s">
+      <c r="F24" s="1" t="s">
         <v>35</v>
       </c>
     </row>
@@ -1014,7 +1014,7 @@
         <f aca="false">FALSE()</f>
         <v>0</v>
       </c>
-      <c r="F25" s="0" t="s">
+      <c r="F25" s="1" t="s">
         <v>35</v>
       </c>
     </row>
@@ -1143,7 +1143,7 @@
       </c>
     </row>
   </sheetData>
-  <conditionalFormatting sqref="C6:E10 C12:E19 C30:E33 C21:E28">
+  <conditionalFormatting sqref="C6:E10 C12:E18 C30:E33 C21:E28 D19:E19">
     <cfRule type="cellIs" priority="2" operator="equal" aboveAverage="0" equalAverage="0" bottom="0" percent="0" rank="0" text="" dxfId="0">
       <formula>0</formula>
     </cfRule>
@@ -1156,6 +1156,11 @@
       <formula>0</formula>
     </cfRule>
   </conditionalFormatting>
+  <conditionalFormatting sqref="C19">
+    <cfRule type="cellIs" priority="5" operator="equal" aboveAverage="0" equalAverage="0" bottom="0" percent="0" rank="0" text="" dxfId="0">
+      <formula>0</formula>
+    </cfRule>
+  </conditionalFormatting>
   <printOptions headings="false" gridLines="false" gridLinesSet="true" horizontalCentered="false" verticalCentered="false"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.511811023622047" footer="0.511811023622047"/>
   <pageSetup paperSize="9" scale="100" fitToWidth="1" fitToHeight="1" pageOrder="downThenOver" orientation="portrait" blackAndWhite="false" draft="false" cellComments="none" horizontalDpi="300" verticalDpi="300" copies="1"/>

</xml_diff>

<commit_message>
weryfikacja przez email gotowa
</commit_message>
<xml_diff>
--- a/sprzatando excel.xlsx
+++ b/sprzatando excel.xlsx
@@ -20,7 +20,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="46" uniqueCount="46">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="45" uniqueCount="45">
   <si>
     <t xml:space="preserve">WYMAGANIA SYSTEMU - Sprzątando</t>
   </si>
@@ -74,9 +74,6 @@
   </si>
   <si>
     <t xml:space="preserve">użytkownik może dodać ogłoszenie-ofertę na sprzątanie (lokalizacja, cena, co sprzątać-&gt;kilka opcji checkbox, opis, czas ważności)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">a</t>
   </si>
   <si>
     <t xml:space="preserve">użytkownik może zgłosić się do realizacji oferty (nie można zgłosić się do swojej oferty)</t>
@@ -674,8 +671,7 @@
         <v>0</v>
       </c>
       <c r="D7" s="1" t="b">
-        <f aca="false">FALSE()</f>
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="E7" s="1" t="b">
         <f aca="false">FALSE()</f>
@@ -683,7 +679,7 @@
       </c>
       <c r="G7" s="3" t="n">
         <f aca="false">COUNTIF(C:E, TRUE())</f>
-        <v>15</v>
+        <v>17</v>
       </c>
     </row>
     <row r="8" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -729,8 +725,7 @@
         <v>0</v>
       </c>
       <c r="D10" s="1" t="b">
-        <f aca="false">FALSE()</f>
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="E10" s="1" t="b">
         <f aca="false">FALSE()</f>
@@ -746,16 +741,14 @@
       </c>
       <c r="G11" s="7" t="n">
         <f aca="false">G7*100/G3</f>
-        <v>60</v>
+        <v>68</v>
       </c>
     </row>
     <row r="12" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A12" s="9" t="s">
         <v>17</v>
       </c>
-      <c r="B12" s="1" t="s">
-        <v>18</v>
-      </c>
+      <c r="B12" s="1"/>
       <c r="C12" s="1" t="b">
         <f aca="false">TRUE()</f>
         <v>1</v>
@@ -771,28 +764,28 @@
     </row>
     <row r="13" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A13" s="9" t="s">
+        <v>18</v>
+      </c>
+      <c r="C13" s="1" t="b">
+        <f aca="false">TRUE()</f>
+        <v>1</v>
+      </c>
+      <c r="D13" s="1" t="b">
+        <f aca="false">FALSE()</f>
+        <v>0</v>
+      </c>
+      <c r="E13" s="1" t="b">
+        <f aca="false">FALSE()</f>
+        <v>0</v>
+      </c>
+      <c r="G13" s="7" t="s">
         <v>19</v>
-      </c>
-      <c r="C13" s="1" t="b">
-        <f aca="false">TRUE()</f>
-        <v>1</v>
-      </c>
-      <c r="D13" s="1" t="b">
-        <f aca="false">FALSE()</f>
-        <v>0</v>
-      </c>
-      <c r="E13" s="1" t="b">
-        <f aca="false">FALSE()</f>
-        <v>0</v>
-      </c>
-      <c r="G13" s="7" t="s">
-        <v>20</v>
       </c>
       <c r="H13" s="7"/>
     </row>
     <row r="14" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A14" s="9" t="s">
-        <v>21</v>
+        <v>20</v>
       </c>
       <c r="C14" s="1" t="b">
         <f aca="false">TRUE()</f>
@@ -810,12 +803,12 @@
         <v>5</v>
       </c>
       <c r="H14" s="7" t="s">
-        <v>22</v>
+        <v>21</v>
       </c>
     </row>
     <row r="15" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A15" s="9" t="s">
-        <v>23</v>
+        <v>22</v>
       </c>
       <c r="C15" s="1" t="b">
         <f aca="false">FALSE()</f>
@@ -833,12 +826,12 @@
         <v>4</v>
       </c>
       <c r="H15" s="7" t="s">
-        <v>24</v>
+        <v>23</v>
       </c>
     </row>
     <row r="16" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A16" s="9" t="s">
-        <v>25</v>
+        <v>24</v>
       </c>
       <c r="C16" s="1" t="b">
         <f aca="false">FALSE()</f>
@@ -856,12 +849,12 @@
         <v>3</v>
       </c>
       <c r="H16" s="7" t="s">
-        <v>26</v>
+        <v>25</v>
       </c>
     </row>
     <row r="17" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A17" s="9" t="s">
-        <v>27</v>
+        <v>26</v>
       </c>
       <c r="C17" s="1" t="b">
         <f aca="false">TRUE()</f>
@@ -879,35 +872,35 @@
         <v>2</v>
       </c>
       <c r="H17" s="7" t="s">
-        <v>28</v>
+        <v>27</v>
       </c>
     </row>
     <row r="18" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A18" s="9" t="s">
+        <v>28</v>
+      </c>
+      <c r="C18" s="1" t="b">
+        <f aca="false">FALSE()</f>
+        <v>0</v>
+      </c>
+      <c r="D18" s="1" t="b">
+        <f aca="false">FALSE()</f>
+        <v>0</v>
+      </c>
+      <c r="E18" s="1" t="b">
+        <f aca="false">FALSE()</f>
+        <v>0</v>
+      </c>
+      <c r="G18" s="7" t="n">
+        <v>1</v>
+      </c>
+      <c r="H18" s="7" t="s">
         <v>29</v>
-      </c>
-      <c r="C18" s="1" t="b">
-        <f aca="false">FALSE()</f>
-        <v>0</v>
-      </c>
-      <c r="D18" s="1" t="b">
-        <f aca="false">FALSE()</f>
-        <v>0</v>
-      </c>
-      <c r="E18" s="1" t="b">
-        <f aca="false">FALSE()</f>
-        <v>0</v>
-      </c>
-      <c r="G18" s="7" t="n">
-        <v>1</v>
-      </c>
-      <c r="H18" s="7" t="s">
-        <v>30</v>
       </c>
     </row>
     <row r="19" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A19" s="9" t="s">
-        <v>31</v>
+        <v>30</v>
       </c>
       <c r="C19" s="1" t="b">
         <f aca="false">FALSE()</f>
@@ -924,12 +917,12 @@
     </row>
     <row r="20" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A20" s="10" t="s">
-        <v>32</v>
+        <v>31</v>
       </c>
     </row>
     <row r="21" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A21" s="11" t="s">
-        <v>33</v>
+        <v>32</v>
       </c>
       <c r="C21" s="1" t="b">
         <f aca="false">TRUE()</f>
@@ -946,7 +939,7 @@
     </row>
     <row r="22" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A22" s="11" t="s">
-        <v>34</v>
+        <v>33</v>
       </c>
       <c r="C22" s="1" t="b">
         <f aca="false">TRUE()</f>
@@ -963,7 +956,7 @@
     </row>
     <row r="23" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A23" s="11" t="s">
-        <v>35</v>
+        <v>34</v>
       </c>
       <c r="C23" s="1" t="b">
         <f aca="false">FALSE()</f>
@@ -981,7 +974,7 @@
     </row>
     <row r="24" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A24" s="11" t="s">
-        <v>36</v>
+        <v>35</v>
       </c>
       <c r="C24" s="1" t="b">
         <f aca="false">FALSE()</f>
@@ -999,7 +992,7 @@
     </row>
     <row r="25" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A25" s="11" t="s">
-        <v>37</v>
+        <v>36</v>
       </c>
       <c r="C25" s="1" t="b">
         <f aca="false">FALSE()</f>
@@ -1017,7 +1010,7 @@
     </row>
     <row r="26" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A26" s="11" t="s">
-        <v>38</v>
+        <v>37</v>
       </c>
       <c r="C26" s="1" t="b">
         <f aca="false">FALSE()</f>
@@ -1034,7 +1027,7 @@
     </row>
     <row r="27" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A27" s="11" t="s">
-        <v>39</v>
+        <v>38</v>
       </c>
       <c r="C27" s="1" t="b">
         <f aca="false">FALSE()</f>
@@ -1051,7 +1044,7 @@
     </row>
     <row r="28" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A28" s="11" t="s">
-        <v>40</v>
+        <v>39</v>
       </c>
       <c r="C28" s="1" t="b">
         <f aca="false">FALSE()</f>
@@ -1068,12 +1061,12 @@
     </row>
     <row r="29" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A29" s="12" t="s">
-        <v>41</v>
+        <v>40</v>
       </c>
     </row>
     <row r="30" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A30" s="13" t="s">
-        <v>42</v>
+        <v>41</v>
       </c>
       <c r="C30" s="1" t="b">
         <f aca="false">FALSE()</f>
@@ -1090,7 +1083,7 @@
     </row>
     <row r="31" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A31" s="13" t="s">
-        <v>43</v>
+        <v>42</v>
       </c>
       <c r="C31" s="1" t="b">
         <f aca="false">FALSE()</f>
@@ -1107,7 +1100,7 @@
     </row>
     <row r="32" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A32" s="13" t="s">
-        <v>44</v>
+        <v>43</v>
       </c>
       <c r="C32" s="1" t="b">
         <f aca="false">FALSE()</f>
@@ -1124,7 +1117,7 @@
     </row>
     <row r="33" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A33" s="13" t="s">
-        <v>45</v>
+        <v>44</v>
       </c>
       <c r="C33" s="1" t="b">
         <f aca="false">FALSE()</f>

</xml_diff>

<commit_message>
panel admin dizła punkt 31 tez
</commit_message>
<xml_diff>
--- a/sprzatando excel.xlsx
+++ b/sprzatando excel.xlsx
@@ -483,37 +483,37 @@
         <a:srgbClr val="000000"/>
       </a:dk1>
       <a:lt1>
-        <a:srgbClr val="ffffff"/>
+        <a:srgbClr val="FFFFFF"/>
       </a:lt1>
       <a:dk2>
-        <a:srgbClr val="44546a"/>
+        <a:srgbClr val="44546A"/>
       </a:dk2>
       <a:lt2>
-        <a:srgbClr val="e7e6e6"/>
+        <a:srgbClr val="E7E6E6"/>
       </a:lt2>
       <a:accent1>
-        <a:srgbClr val="5b9bd5"/>
+        <a:srgbClr val="5B9BD5"/>
       </a:accent1>
       <a:accent2>
-        <a:srgbClr val="ed7d31"/>
+        <a:srgbClr val="ED7D31"/>
       </a:accent2>
       <a:accent3>
-        <a:srgbClr val="a5a5a5"/>
+        <a:srgbClr val="A5A5A5"/>
       </a:accent3>
       <a:accent4>
-        <a:srgbClr val="ffc000"/>
+        <a:srgbClr val="FFC000"/>
       </a:accent4>
       <a:accent5>
-        <a:srgbClr val="4472c4"/>
+        <a:srgbClr val="4472C4"/>
       </a:accent5>
       <a:accent6>
-        <a:srgbClr val="70ad47"/>
+        <a:srgbClr val="70AD47"/>
       </a:accent6>
       <a:hlink>
-        <a:srgbClr val="0563c1"/>
+        <a:srgbClr val="0563C1"/>
       </a:hlink>
       <a:folHlink>
-        <a:srgbClr val="954f72"/>
+        <a:srgbClr val="954F72"/>
       </a:folHlink>
     </a:clrScheme>
     <a:fontScheme name="Office">
@@ -671,6 +671,7 @@
         <v>0</v>
       </c>
       <c r="D7" s="1" t="b">
+        <f aca="false">TRUE()</f>
         <v>1</v>
       </c>
       <c r="E7" s="1" t="b">
@@ -679,7 +680,7 @@
       </c>
       <c r="G7" s="3" t="n">
         <f aca="false">COUNTIF(C:E, TRUE())</f>
-        <v>17</v>
+        <v>18</v>
       </c>
     </row>
     <row r="8" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -725,6 +726,7 @@
         <v>0</v>
       </c>
       <c r="D10" s="1" t="b">
+        <f aca="false">TRUE()</f>
         <v>1</v>
       </c>
       <c r="E10" s="1" t="b">
@@ -741,7 +743,7 @@
       </c>
       <c r="G11" s="7" t="n">
         <f aca="false">G7*100/G3</f>
-        <v>68</v>
+        <v>72</v>
       </c>
     </row>
     <row r="12" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -1094,8 +1096,8 @@
         <v>0</v>
       </c>
       <c r="E31" s="1" t="b">
-        <f aca="false">FALSE()</f>
-        <v>0</v>
+        <f aca="false">TRUE()</f>
+        <v>1</v>
       </c>
     </row>
     <row r="32" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">

</xml_diff>

<commit_message>
naprawia zmiany emialu i sql
</commit_message>
<xml_diff>
--- a/sprzatando excel.xlsx
+++ b/sprzatando excel.xlsx
@@ -483,37 +483,37 @@
         <a:srgbClr val="000000"/>
       </a:dk1>
       <a:lt1>
-        <a:srgbClr val="FFFFFF"/>
+        <a:srgbClr val="ffffff"/>
       </a:lt1>
       <a:dk2>
-        <a:srgbClr val="44546A"/>
+        <a:srgbClr val="44546a"/>
       </a:dk2>
       <a:lt2>
-        <a:srgbClr val="E7E6E6"/>
+        <a:srgbClr val="e7e6e6"/>
       </a:lt2>
       <a:accent1>
-        <a:srgbClr val="5B9BD5"/>
+        <a:srgbClr val="5b9bd5"/>
       </a:accent1>
       <a:accent2>
-        <a:srgbClr val="ED7D31"/>
+        <a:srgbClr val="ed7d31"/>
       </a:accent2>
       <a:accent3>
-        <a:srgbClr val="A5A5A5"/>
+        <a:srgbClr val="a5a5a5"/>
       </a:accent3>
       <a:accent4>
-        <a:srgbClr val="FFC000"/>
+        <a:srgbClr val="ffc000"/>
       </a:accent4>
       <a:accent5>
-        <a:srgbClr val="4472C4"/>
+        <a:srgbClr val="4472c4"/>
       </a:accent5>
       <a:accent6>
-        <a:srgbClr val="70AD47"/>
+        <a:srgbClr val="70ad47"/>
       </a:accent6>
       <a:hlink>
-        <a:srgbClr val="0563C1"/>
+        <a:srgbClr val="0563c1"/>
       </a:hlink>
       <a:folHlink>
-        <a:srgbClr val="954F72"/>
+        <a:srgbClr val="954f72"/>
       </a:folHlink>
     </a:clrScheme>
     <a:fontScheme name="Office">

</xml_diff>